<commit_message>
Integrerer nye 2025-resultater: Oppdaterte rekorder og nye svømmere
</commit_message>
<xml_diff>
--- a/EndResult/100m Butterfly.xlsx
+++ b/EndResult/100m Butterfly.xlsx
@@ -1549,7 +1549,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Amanda Husan Ehrnholm</t>
+          <t>Sanna Josefin Husan Ehrnholm</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1562,12 +1562,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16.01.2016</t>
+          <t>03.12.2016</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Trondheim</t>
+          <t>Stjørdal</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1584,7 +1584,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sanna Josefin Husan Ehrnholm</t>
+          <t>Amanda Husan Ehrnholm</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1597,12 +1597,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>03.12.2016</t>
+          <t>16.01.2016</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Stjørdal</t>
+          <t>Trondheim</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">

</xml_diff>